<commit_message>
Updated assigned lab sections to reflect changes made during add-drop week
</commit_message>
<xml_diff>
--- a/Office Hours Spreadsheet.xlsx
+++ b/Office Hours Spreadsheet.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="124">
   <si>
     <t>This sheet will be used to track office hours for PTs. 
 Similar to last semester, there are only 2 PTs in the PTC Monday through Wednesday from 8-10 am, 3 PTs at 8-9 am on Thursday.
@@ -38,6 +38,9 @@
     <t>TUESDAY</t>
   </si>
   <si>
+    <t>THURSDAY</t>
+  </si>
+  <si>
     <t>WEDNESDAY</t>
   </si>
   <si>
@@ -50,7 +53,7 @@
     <t>Jianwei Gao</t>
   </si>
   <si>
-    <t>THURSDAY</t>
+    <t>Ross Moore</t>
   </si>
   <si>
     <t>Admin Block</t>
@@ -68,27 +71,27 @@
     <t>Dunsin Komolafe</t>
   </si>
   <si>
+    <t>9:30 - 10:00</t>
+  </si>
+  <si>
     <t>Isabella Chan Tack</t>
   </si>
   <si>
-    <t>9:30 - 10:00</t>
-  </si>
-  <si>
     <t>Casey Roper</t>
   </si>
   <si>
     <t>10:00 - 10:30</t>
   </si>
   <si>
-    <t>Tejas Kalpathi</t>
-  </si>
-  <si>
     <t>Orlando Haye</t>
   </si>
   <si>
     <t>10:30 - 11:00</t>
   </si>
   <si>
+    <t>Sawyer Nguyen</t>
+  </si>
+  <si>
     <t>Joyce You</t>
   </si>
   <si>
@@ -98,232 +101,226 @@
     <t>11:30 - 12:00</t>
   </si>
   <si>
+    <t>Amin Karic</t>
+  </si>
+  <si>
     <t>12:00 - 12:30</t>
   </si>
   <si>
+    <t>Parker Wolski</t>
+  </si>
+  <si>
+    <t>Shruti Oruganti</t>
+  </si>
+  <si>
+    <t>12:30 - 1:00</t>
+  </si>
+  <si>
+    <t>Jared White</t>
+  </si>
+  <si>
+    <t>Elisa Bibb</t>
+  </si>
+  <si>
+    <t>Colin Xu</t>
+  </si>
+  <si>
+    <t>Ethan Kigotho</t>
+  </si>
+  <si>
+    <t>1:00 - 1:30</t>
+  </si>
+  <si>
+    <t>William Stone</t>
+  </si>
+  <si>
+    <t>1:30 - 2:00</t>
+  </si>
+  <si>
+    <t>Angela Yue</t>
+  </si>
+  <si>
+    <t>2:00 - 2:30</t>
+  </si>
+  <si>
+    <t>Kesha Patel</t>
+  </si>
+  <si>
+    <t>Saachi Jain</t>
+  </si>
+  <si>
+    <t>2:30 - 3:00</t>
+  </si>
+  <si>
+    <t>Srihari Yechangunja</t>
+  </si>
+  <si>
+    <t>3:00 - 3:30</t>
+  </si>
+  <si>
+    <t>3:30 - 4:00</t>
+  </si>
+  <si>
+    <t>4:00 - 4:30</t>
+  </si>
+  <si>
+    <t>Sai Sudarshan Barath</t>
+  </si>
+  <si>
+    <t>Nishit Aggarwal</t>
+  </si>
+  <si>
+    <t>Kaushik Nagarajan</t>
+  </si>
+  <si>
+    <t>4:30 - 5:00</t>
+  </si>
+  <si>
     <t>Malakai Coleman</t>
   </si>
   <si>
-    <t>Sawyer Nguyen</t>
-  </si>
-  <si>
-    <t>Ross Moore</t>
-  </si>
-  <si>
-    <t>Ethan Kigotho</t>
-  </si>
-  <si>
-    <t>Shruti Oruganti</t>
-  </si>
-  <si>
-    <t>12:30 - 1:00</t>
-  </si>
-  <si>
-    <t>Elisa Bibb</t>
-  </si>
-  <si>
-    <t>1:00 - 1:30</t>
-  </si>
-  <si>
-    <t>Angela Yue</t>
-  </si>
-  <si>
-    <t>Colin Xu</t>
-  </si>
-  <si>
-    <t>1:30 - 2:00</t>
-  </si>
-  <si>
-    <t>Sai Sudarshan Barath</t>
-  </si>
-  <si>
-    <t>2:00 - 2:30</t>
-  </si>
-  <si>
-    <t>Kesha Patel</t>
-  </si>
-  <si>
-    <t>Saachi Jain</t>
-  </si>
-  <si>
-    <t>2:30 - 3:00</t>
-  </si>
-  <si>
-    <t>Srihari Yechangunja</t>
-  </si>
-  <si>
-    <t>3:00 - 3:30</t>
-  </si>
-  <si>
-    <t>3:30 - 4:00</t>
-  </si>
-  <si>
-    <t>4:00 - 4:30</t>
-  </si>
-  <si>
-    <t>Kaushik Nagarajan</t>
-  </si>
-  <si>
-    <t>4:30 - 5:00</t>
-  </si>
-  <si>
-    <t>Jared White</t>
-  </si>
-  <si>
-    <t>Amin Karic</t>
-  </si>
-  <si>
-    <t>Parker Wolski</t>
-  </si>
-  <si>
-    <t>William Stone</t>
+    <t>FRIDAY</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>First</t>
+  </si>
+  <si>
+    <t>120 Review</t>
+  </si>
+  <si>
+    <t>Last</t>
+  </si>
+  <si>
+    <t>Concat</t>
+  </si>
+  <si>
+    <t>⠀⠀</t>
+  </si>
+  <si>
+    <t>⠀⠀⠀</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Block</t>
+  </si>
+  <si>
+    <t>221 Review</t>
+  </si>
+  <si>
+    <t>222 Review</t>
+  </si>
+  <si>
+    <t>313 Review</t>
+  </si>
+  <si>
+    <t>Nishit</t>
+  </si>
+  <si>
+    <t>Aggarwal</t>
+  </si>
+  <si>
+    <t>Andrew</t>
+  </si>
+  <si>
+    <t>Bae</t>
+  </si>
+  <si>
+    <t>312 Review</t>
+  </si>
+  <si>
+    <t>Sai Sudarshan</t>
+  </si>
+  <si>
+    <t>Barath</t>
+  </si>
+  <si>
+    <t>314 Review</t>
+  </si>
+  <si>
+    <t>Elisa</t>
+  </si>
+  <si>
+    <t>Bibb</t>
+  </si>
+  <si>
+    <t>Isabella</t>
+  </si>
+  <si>
+    <t>Chan Tack</t>
+  </si>
+  <si>
+    <t>Malakai</t>
+  </si>
+  <si>
+    <t>Coleman</t>
+  </si>
+  <si>
+    <t>Johnny</t>
+  </si>
+  <si>
+    <t>Figueroa</t>
+  </si>
+  <si>
+    <t>Jianwei</t>
+  </si>
+  <si>
+    <t>Gao</t>
+  </si>
+  <si>
+    <t>Orlando</t>
+  </si>
+  <si>
+    <t>Haye</t>
+  </si>
+  <si>
+    <t>Saachi</t>
+  </si>
+  <si>
+    <t>Jain</t>
+  </si>
+  <si>
+    <t>Tejas</t>
+  </si>
+  <si>
+    <t>Kalpathi</t>
+  </si>
+  <si>
+    <t>Amin</t>
+  </si>
+  <si>
+    <t>Karic</t>
+  </si>
+  <si>
+    <t>Ethan</t>
+  </si>
+  <si>
+    <t>Kigotho</t>
+  </si>
+  <si>
+    <t>Dunsin</t>
+  </si>
+  <si>
+    <t>Komolafe</t>
+  </si>
+  <si>
+    <t>Ross</t>
+  </si>
+  <si>
+    <t>Moore</t>
+  </si>
+  <si>
+    <t>Kaushik</t>
+  </si>
+  <si>
+    <t>Nagarajan</t>
   </si>
   <si>
     <t>Johnny Figueroa</t>
-  </si>
-  <si>
-    <t>Nishit Aggarwal</t>
-  </si>
-  <si>
-    <t>FRIDAY</t>
-  </si>
-  <si>
-    <t>Sunday</t>
-  </si>
-  <si>
-    <t>120 Review</t>
-  </si>
-  <si>
-    <t>First</t>
-  </si>
-  <si>
-    <t>Last</t>
-  </si>
-  <si>
-    <t>Concat</t>
-  </si>
-  <si>
-    <t>⠀⠀</t>
-  </si>
-  <si>
-    <t>221 Review</t>
-  </si>
-  <si>
-    <t>⠀⠀⠀</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>Block</t>
-  </si>
-  <si>
-    <t>222 Review</t>
-  </si>
-  <si>
-    <t>313 Review</t>
-  </si>
-  <si>
-    <t>312 Review</t>
-  </si>
-  <si>
-    <t>314 Review</t>
-  </si>
-  <si>
-    <t>Nishit</t>
-  </si>
-  <si>
-    <t>Aggarwal</t>
-  </si>
-  <si>
-    <t>Andrew</t>
-  </si>
-  <si>
-    <t>Bae</t>
-  </si>
-  <si>
-    <t>Sai Sudarshan</t>
-  </si>
-  <si>
-    <t>Barath</t>
-  </si>
-  <si>
-    <t>Elisa</t>
-  </si>
-  <si>
-    <t>Bibb</t>
-  </si>
-  <si>
-    <t>Isabella</t>
-  </si>
-  <si>
-    <t>Chan Tack</t>
-  </si>
-  <si>
-    <t>Malakai</t>
-  </si>
-  <si>
-    <t>Coleman</t>
-  </si>
-  <si>
-    <t>Johnny</t>
-  </si>
-  <si>
-    <t>Figueroa</t>
-  </si>
-  <si>
-    <t>Jianwei</t>
-  </si>
-  <si>
-    <t>Gao</t>
-  </si>
-  <si>
-    <t>Orlando</t>
-  </si>
-  <si>
-    <t>Haye</t>
-  </si>
-  <si>
-    <t>Saachi</t>
-  </si>
-  <si>
-    <t>Jain</t>
-  </si>
-  <si>
-    <t>Tejas</t>
-  </si>
-  <si>
-    <t>Kalpathi</t>
-  </si>
-  <si>
-    <t>Amin</t>
-  </si>
-  <si>
-    <t>Karic</t>
-  </si>
-  <si>
-    <t>Ethan</t>
-  </si>
-  <si>
-    <t>Kigotho</t>
-  </si>
-  <si>
-    <t>Dunsin</t>
-  </si>
-  <si>
-    <t>Komolafe</t>
-  </si>
-  <si>
-    <t>Ross</t>
-  </si>
-  <si>
-    <t>Moore</t>
-  </si>
-  <si>
-    <t>Kaushik</t>
-  </si>
-  <si>
-    <t>Nagarajan</t>
   </si>
   <si>
     <t>Sawyer</t>
@@ -415,6 +412,10 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="14.0"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <sz val="12.0"/>
       <name val="Lato"/>
     </font>
@@ -423,10 +424,6 @@
       <name val="Lato"/>
     </font>
     <font/>
-    <font>
-      <sz val="14.0"/>
-      <name val="Calibri"/>
-    </font>
     <font>
       <sz val="12.0"/>
       <color rgb="FF181A1B"/>
@@ -560,48 +557,48 @@
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="2" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="2" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -613,7 +610,7 @@
     <xf borderId="0" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="8" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -674,7 +671,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="522.75" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -696,47 +693,47 @@
   </cols>
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="5"/>
     </row>
     <row r="2" ht="24.0" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" ht="24.0" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" ht="24.0" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
@@ -744,25 +741,25 @@
         <v>14</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -770,90 +767,90 @@
         <v>19</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>25</v>
-      </c>
       <c r="D7" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>20</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D10" s="9"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>30</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>18</v>
@@ -861,13 +858,13 @@
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>18</v>
@@ -875,52 +872,58 @@
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="9"/>
+        <v>45</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
+      <c r="D16" s="7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
+      <c r="D17" s="7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
@@ -954,47 +957,47 @@
   </cols>
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="5"/>
     </row>
     <row r="2" ht="24.0" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" ht="24.0" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" ht="24.0" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
@@ -1002,27 +1005,27 @@
         <v>14</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -1033,170 +1036,174 @@
         <v>18</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D14" s="7"/>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>38</v>
-      </c>
       <c r="D15" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7" t="s">
-        <v>40</v>
-      </c>
       <c r="D16" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>35</v>
-      </c>
       <c r="C19" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1228,49 +1235,51 @@
   </cols>
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="4"/>
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="5"/>
     </row>
     <row r="2" ht="24.0" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" ht="24.0" customHeight="1">
       <c r="A3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>9</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="8" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
@@ -1278,25 +1287,27 @@
         <v>14</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="7"/>
+        <v>17</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="C6" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -1304,91 +1315,91 @@
         <v>19</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>20</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>18</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>18</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>30</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>30</v>
@@ -1397,13 +1408,13 @@
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>30</v>
@@ -1411,11 +1422,11 @@
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>30</v>
@@ -1423,13 +1434,13 @@
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>30</v>
@@ -1437,13 +1448,13 @@
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>30</v>
@@ -1451,20 +1462,20 @@
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
@@ -1498,55 +1509,55 @@
   </cols>
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="5"/>
     </row>
     <row r="2" ht="24.0" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" ht="24.0" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" ht="24.0" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
@@ -1554,25 +1565,25 @@
         <v>14</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>15</v>
-      </c>
       <c r="C6" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
@@ -1582,191 +1593,195 @@
         <v>19</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>18</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="D7" s="7"/>
       <c r="E7" s="7"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>18</v>
-      </c>
+      <c r="D8" s="7"/>
       <c r="E8" s="7" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>31</v>
+      </c>
       <c r="E11" s="7" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>30</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>31</v>
+      </c>
       <c r="E12" s="7" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>30</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>31</v>
+      </c>
       <c r="E13" s="7" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>38</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
       <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
+      <c r="E14" s="7" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>38</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
       <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
+      <c r="E15" s="7" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="7"/>
+        <v>12</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
+      <c r="E16" s="7" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="7"/>
+        <v>12</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>39</v>
+      </c>
       <c r="D17" s="7"/>
       <c r="E17" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>35</v>
-      </c>
       <c r="D19" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E19" s="7"/>
     </row>
@@ -1799,24 +1814,24 @@
   </cols>
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="4"/>
+      <c r="A1" s="2"/>
+      <c r="B1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" ht="24.0" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
@@ -1824,33 +1839,31 @@
     </row>
     <row r="3" ht="24.0" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>51</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D3" s="7"/>
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7" t="s">
         <v>30</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F4" s="7"/>
     </row>
@@ -1859,35 +1872,35 @@
         <v>14</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7" t="s">
         <v>30</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F5" s="7"/>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>30</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -1895,216 +1908,222 @@
         <v>19</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>30</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>18</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>18</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>27</v>
-      </c>
       <c r="F11" s="7" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D12" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>27</v>
-      </c>
       <c r="F12" s="7" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="7"/>
+        <v>47</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="D13" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="7" t="s">
-        <v>27</v>
-      </c>
       <c r="F13" s="7" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>32</v>
-      </c>
       <c r="E14" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>31</v>
+      </c>
       <c r="C15" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>33</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="E15" s="7"/>
       <c r="F15" s="7" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="7"/>
+        <v>42</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>31</v>
+      </c>
       <c r="C16" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>33</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="E16" s="7"/>
       <c r="F16" s="7" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="7"/>
+        <v>43</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>31</v>
+      </c>
       <c r="C17" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="7" t="s">
-        <v>50</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="7"/>
+        <v>44</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>31</v>
+      </c>
       <c r="C18" s="7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
@@ -2112,12 +2131,12 @@
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7" t="s">
-        <v>24</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
@@ -2152,77 +2171,77 @@
   </cols>
   <sheetData>
     <row r="1" ht="36.0" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="5"/>
+    </row>
+    <row r="2" ht="24.0" customHeight="1">
+      <c r="A2" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="4"/>
-    </row>
-    <row r="2" ht="24.0" customHeight="1">
-      <c r="A2" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="4"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" ht="24.0" customHeight="1">
       <c r="A3" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="B3" s="4"/>
+        <v>60</v>
+      </c>
+      <c r="B3" s="5"/>
       <c r="C3" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="4"/>
+        <v>61</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" ht="24.0" customHeight="1">
       <c r="A4" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="B4" s="4"/>
+        <v>62</v>
+      </c>
+      <c r="B4" s="5"/>
       <c r="C4" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="D4" s="4"/>
+        <v>67</v>
+      </c>
+      <c r="D4" s="5"/>
       <c r="E4" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="F4" s="4"/>
+        <v>70</v>
+      </c>
+      <c r="F4" s="5"/>
     </row>
     <row r="5" ht="24.0" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" ht="24.0" customHeight="1">
       <c r="A6" s="17" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C6" s="18"/>
       <c r="D6" s="18"/>
@@ -2231,10 +2250,10 @@
     </row>
     <row r="7" ht="24.0" customHeight="1">
       <c r="A7" s="17" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="C7" s="18"/>
       <c r="D7" s="18"/>
@@ -2243,71 +2262,75 @@
     </row>
     <row r="8" ht="24.0" customHeight="1">
       <c r="A8" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="D8" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>44</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
     </row>
     <row r="9" ht="24.0" customHeight="1">
       <c r="A9" s="19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
     </row>
     <row r="10" ht="24.0" customHeight="1">
       <c r="A10" s="20" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" ht="24.0" customHeight="1">
       <c r="A11" s="20" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
+        <v>16</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" s="20" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="12" ht="24.0" customHeight="1">
       <c r="A12" s="7"/>
@@ -2454,30 +2477,30 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="12" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="B2" s="13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="14" t="s">
+    <row r="3">
+      <c r="A3" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>62</v>
+      <c r="B3" s="13" t="s">
+        <v>59</v>
       </c>
       <c r="C3" t="str">
         <f t="shared" ref="C3:C32" si="1">TEXTJOIN(" ", True, A3, B3)</f>
@@ -2485,11 +2508,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>68</v>
+      <c r="A4" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>64</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="1"/>
@@ -2497,11 +2520,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>70</v>
+      <c r="A5" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>66</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="1"/>
@@ -2509,11 +2532,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>72</v>
+      <c r="A6" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>69</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="1"/>
@@ -2521,11 +2544,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>74</v>
+      <c r="A7" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>72</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="1"/>
@@ -2533,11 +2556,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>76</v>
+      <c r="A8" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="1"/>
@@ -2545,11 +2568,11 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>78</v>
+      <c r="A9" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>76</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="1"/>
@@ -2557,11 +2580,11 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>80</v>
+      <c r="A10" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>78</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="1"/>
@@ -2569,11 +2592,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>82</v>
+      <c r="A11" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>80</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="1"/>
@@ -2581,11 +2604,11 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>84</v>
+      <c r="A12" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>82</v>
       </c>
       <c r="C12" t="str">
         <f t="shared" si="1"/>
@@ -2593,11 +2616,11 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>86</v>
+      <c r="A13" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>84</v>
       </c>
       <c r="C13" t="str">
         <f t="shared" si="1"/>
@@ -2605,11 +2628,11 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>88</v>
+      <c r="A14" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>86</v>
       </c>
       <c r="C14" t="str">
         <f t="shared" si="1"/>
@@ -2617,11 +2640,11 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>90</v>
+      <c r="A15" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>88</v>
       </c>
       <c r="C15" t="str">
         <f t="shared" si="1"/>
@@ -2629,11 +2652,11 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>92</v>
+      <c r="A16" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>90</v>
       </c>
       <c r="C16" t="str">
         <f t="shared" si="1"/>
@@ -2641,11 +2664,11 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>94</v>
+      <c r="A17" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>92</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="1"/>
@@ -2653,11 +2676,11 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>96</v>
+      <c r="A18" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>94</v>
       </c>
       <c r="C18" t="str">
         <f t="shared" si="1"/>
@@ -2665,11 +2688,11 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>98</v>
+      <c r="A19" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>96</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="1"/>
@@ -2677,11 +2700,11 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B20" s="13" t="s">
         <v>99</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>100</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="1"/>
@@ -2689,11 +2712,11 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="13" t="s">
         <v>101</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>102</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="1"/>
@@ -2701,11 +2724,11 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" s="13" t="s">
         <v>103</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>104</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="1"/>
@@ -2713,11 +2736,11 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" s="13" t="s">
         <v>105</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>106</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" si="1"/>
@@ -2725,11 +2748,11 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="B24" s="13" t="s">
         <v>107</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>108</v>
       </c>
       <c r="C24" t="str">
         <f t="shared" si="1"/>
@@ -2737,11 +2760,11 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B25" s="13" t="s">
         <v>109</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>110</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="1"/>
@@ -2749,11 +2772,11 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="13" t="s">
         <v>111</v>
-      </c>
-      <c r="B26" s="14" t="s">
-        <v>112</v>
       </c>
       <c r="C26" t="str">
         <f t="shared" si="1"/>
@@ -2761,11 +2784,11 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="s">
+      <c r="A27" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" s="13" t="s">
         <v>113</v>
-      </c>
-      <c r="B27" s="14" t="s">
-        <v>114</v>
       </c>
       <c r="C27" t="str">
         <f t="shared" si="1"/>
@@ -2773,11 +2796,11 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="B28" s="13" t="s">
         <v>115</v>
-      </c>
-      <c r="B28" s="14" t="s">
-        <v>116</v>
       </c>
       <c r="C28" t="str">
         <f t="shared" si="1"/>
@@ -2785,11 +2808,11 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="B29" s="13" t="s">
         <v>117</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>118</v>
       </c>
       <c r="C29" t="str">
         <f t="shared" si="1"/>
@@ -2797,11 +2820,11 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B30" s="13" t="s">
         <v>119</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>120</v>
       </c>
       <c r="C30" t="str">
         <f t="shared" si="1"/>
@@ -2809,11 +2832,11 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="s">
+      <c r="A31" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>121</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>122</v>
       </c>
       <c r="C31" t="str">
         <f t="shared" si="1"/>
@@ -2821,11 +2844,11 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="14" t="s">
+      <c r="A32" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="B32" s="13" t="s">
         <v>123</v>
-      </c>
-      <c r="B32" s="14" t="s">
-        <v>124</v>
       </c>
       <c r="C32" t="str">
         <f t="shared" si="1"/>

</xml_diff>